<commit_message>
Checklist log update 2026-07-29T23:17:55.936Z
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -815,9 +815,399 @@
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B17" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C17" t="str">
+        <v>test</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="F17" t="str">
+        <v>N</v>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B18" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C18" t="str">
+        <v>test</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Check Grecon Tank is On "operational Level</v>
+      </c>
+      <c r="F18" t="str">
+        <v>N</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B19" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C19" t="str">
+        <v>test</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Check Water Sprayers are Functioning Correctly</v>
+      </c>
+      <c r="F19" t="str">
+        <v>N</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B20" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C20" t="str">
+        <v>test</v>
+      </c>
+      <c r="D20" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Check Mill Adjustment Sheet is Up to Date</v>
+      </c>
+      <c r="F20" t="str">
+        <v>N</v>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B21" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C21" t="str">
+        <v>test</v>
+      </c>
+      <c r="D21" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Purge Mills with 200 pumps each @ 9 AM</v>
+      </c>
+      <c r="F21" t="str">
+        <v>N</v>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B22" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C22" t="str">
+        <v>test</v>
+      </c>
+      <c r="D22" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Purge Mills with 200 pumps each @ 3 PM</v>
+      </c>
+      <c r="F22" t="str">
+        <v>N</v>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B23" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C23" t="str">
+        <v>test</v>
+      </c>
+      <c r="D23" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Purge Mills with 200 pumps each @ 9 PM</v>
+      </c>
+      <c r="F23" t="str">
+        <v>N</v>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B24" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C24" t="str">
+        <v>test</v>
+      </c>
+      <c r="D24" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Purge Mills with 200 pumps each @ 3 AM</v>
+      </c>
+      <c r="F24" t="str">
+        <v>N</v>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B25" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C25" t="str">
+        <v>test</v>
+      </c>
+      <c r="D25" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Inspect &amp; Clean Steam Vent @ 530 PM</v>
+      </c>
+      <c r="F25" t="str">
+        <v>N</v>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B26" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C26" t="str">
+        <v>test</v>
+      </c>
+      <c r="D26" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Inspect &amp; Clean Steam Vent @ 530 AM</v>
+      </c>
+      <c r="F26" t="str">
+        <v>N</v>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B27" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C27" t="str">
+        <v>test</v>
+      </c>
+      <c r="D27" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Empty Drop Box At End of Shift</v>
+      </c>
+      <c r="F27" t="str">
+        <v>N</v>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B28" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C28" t="str">
+        <v>test</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="E28" t="str">
+        <v xml:space="preserve">Deep Clean Around Mills </v>
+      </c>
+      <c r="F28" t="str">
+        <v>N</v>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B29" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C29" t="str">
+        <v>test</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Clean Diverters / Shavings 1 into 2 Transition</v>
+      </c>
+      <c r="F29" t="str">
+        <v>N</v>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C30" t="str">
+        <v>test</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Check Dinking Water Tank Level</v>
+      </c>
+      <c r="F30" t="str">
+        <v>N</v>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="B31" t="str">
+        <v>09:17:55</v>
+      </c>
+      <c r="C31" t="str">
+        <v>test</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Empty All Bins And Wheel Barrows</v>
+      </c>
+      <c r="F31" t="str">
+        <v>N</v>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-08-06T21:18:27.839Z
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:J45"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1298,9 +1298,457 @@
         <v>S-ms6r15uy-omydl</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C32" t="str">
+        <v>07:17</v>
+      </c>
+      <c r="D32" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
+      <c r="I32" t="str">
+        <v/>
+      </c>
+      <c r="J32" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C33" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D33" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="G33" t="str">
+        <v>N</v>
+      </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C34" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D34" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="G34" t="str">
+        <v>N</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C35" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D35" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="G35" t="str">
+        <v>N</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C36" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D36" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="G36" t="str">
+        <v>N</v>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C37" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D37" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E37" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="G37" t="str">
+        <v>N</v>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C38" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D38" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E38" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="G38" t="str">
+        <v>N</v>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C39" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D39" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E39" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="G39" t="str">
+        <v>N</v>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C40" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D40" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E40" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="G40" t="str">
+        <v>N</v>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+      <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C41" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D41" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E41" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="G41" t="str">
+        <v>N</v>
+      </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
+      <c r="I41" t="str">
+        <v/>
+      </c>
+      <c r="J41" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C42" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D42" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="G42" t="str">
+        <v>N</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C43" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D43" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="G43" t="str">
+        <v>N</v>
+      </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C44" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D44" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="G44" t="str">
+        <v>N</v>
+      </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
+      <c r="I44" t="str">
+        <v/>
+      </c>
+      <c r="J44" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C45" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D45" t="str">
+        <v>chris</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="G45" t="str">
+        <v>N</v>
+      </c>
+      <c r="H45" t="str">
+        <v/>
+      </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45" t="str">
+        <v>S-msi0gawj-ya6co</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J45"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>